<commit_message>
fix some formatting on bank overview
</commit_message>
<xml_diff>
--- a/banks/ALDERMORE FINANCIALS.xlsx
+++ b/banks/ALDERMORE FINANCIALS.xlsx
@@ -2126,15 +2126,40 @@
       <c r="M6" s="5" t="n">
         <v>5583.2</v>
       </c>
-      <c r="N6" s="5" t="n"/>
-      <c r="O6" s="5" t="n"/>
-      <c r="P6" s="5" t="n"/>
-      <c r="Q6" s="5" t="n"/>
-      <c r="R6" s="5" t="n"/>
+      <c r="N6" s="5" t="n">
+        <v>4194.3</v>
+      </c>
+      <c r="O6" s="5" t="n">
+        <v>2519.6</v>
+      </c>
+      <c r="P6" s="5" t="n">
+        <v>1554.1</v>
+      </c>
+      <c r="Q6" s="5" t="n">
+        <v>752.3</v>
+      </c>
+      <c r="R6" s="5" t="n">
+        <v>294.7</v>
+      </c>
       <c r="U6" t="inlineStr">
         <is>
           <t>Total assets</t>
         </is>
+      </c>
+      <c r="V6" t="n">
+        <v>294.7</v>
+      </c>
+      <c r="W6" t="n">
+        <v>752.3</v>
+      </c>
+      <c r="X6" t="n">
+        <v>1554.1</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>2519.6</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>4194.3</v>
       </c>
       <c r="AA6" t="n">
         <v>5583.2</v>
@@ -2248,15 +2273,40 @@
       <c r="M7" s="5" t="n">
         <v>4801.1</v>
       </c>
-      <c r="N7" s="5" t="n"/>
-      <c r="O7" s="5" t="n"/>
-      <c r="P7" s="5" t="n"/>
-      <c r="Q7" s="5" t="n"/>
-      <c r="R7" s="5" t="n"/>
+      <c r="N7" s="5" t="n">
+        <v>3370.8</v>
+      </c>
+      <c r="O7" s="5" t="n">
+        <v>2059.6</v>
+      </c>
+      <c r="P7" s="5" t="n">
+        <v>1160.4</v>
+      </c>
+      <c r="Q7" s="5" t="n">
+        <v>475</v>
+      </c>
+      <c r="R7" s="5" t="n">
+        <v>160.6</v>
+      </c>
       <c r="U7" t="inlineStr">
         <is>
           <t>Loans and advances to customers</t>
         </is>
+      </c>
+      <c r="V7" t="n">
+        <v>160.6</v>
+      </c>
+      <c r="W7" t="n">
+        <v>475</v>
+      </c>
+      <c r="X7" t="n">
+        <v>1160.4</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>2059.6</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>3370.8</v>
       </c>
       <c r="AA7" t="n">
         <v>4801.1</v>
@@ -2370,15 +2420,40 @@
       <c r="M8" s="5" t="n">
         <v>4459</v>
       </c>
-      <c r="N8" s="5" t="n"/>
-      <c r="O8" s="5" t="n"/>
-      <c r="P8" s="5" t="n"/>
-      <c r="Q8" s="5" t="n"/>
-      <c r="R8" s="5" t="n"/>
+      <c r="N8" s="5" t="n">
+        <v>3444.4</v>
+      </c>
+      <c r="O8" s="5" t="n">
+        <v>2141.2</v>
+      </c>
+      <c r="P8" s="5" t="n">
+        <v>1347.5</v>
+      </c>
+      <c r="Q8" s="5" t="n">
+        <v>634.7</v>
+      </c>
+      <c r="R8" s="5" t="n">
+        <v>229.6</v>
+      </c>
       <c r="U8" t="inlineStr">
         <is>
           <t>Customers' accounts</t>
         </is>
+      </c>
+      <c r="V8" t="n">
+        <v>229.6</v>
+      </c>
+      <c r="W8" t="n">
+        <v>634.7</v>
+      </c>
+      <c r="X8" t="n">
+        <v>1347.5</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>2141.2</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>3444.4</v>
       </c>
       <c r="AA8" t="n">
         <v>4459</v>
@@ -2492,15 +2567,40 @@
       <c r="M9" s="5" t="n">
         <v>374.8</v>
       </c>
-      <c r="N9" s="5" t="n"/>
-      <c r="O9" s="5" t="n"/>
-      <c r="P9" s="5" t="n"/>
-      <c r="Q9" s="5" t="n"/>
-      <c r="R9" s="5" t="n"/>
+      <c r="N9" s="5" t="n">
+        <v>257.4</v>
+      </c>
+      <c r="O9" s="5" t="n">
+        <v>172.3</v>
+      </c>
+      <c r="P9" s="5" t="n">
+        <v>166.1</v>
+      </c>
+      <c r="Q9" s="5" t="n">
+        <v>91.59999999999999</v>
+      </c>
+      <c r="R9" s="5" t="n">
+        <v>53.1</v>
+      </c>
       <c r="U9" t="inlineStr">
         <is>
           <t>Total equity</t>
         </is>
+      </c>
+      <c r="V9" t="n">
+        <v>53.1</v>
+      </c>
+      <c r="W9" t="n">
+        <v>91.59999999999999</v>
+      </c>
+      <c r="X9" t="n">
+        <v>166.1</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>172.3</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>257.4</v>
       </c>
       <c r="AA9" t="n">
         <v>374.8</v>
@@ -2831,15 +2931,40 @@
       <c r="M13" s="5" t="n">
         <v>166.1</v>
       </c>
-      <c r="N13" s="5" t="n"/>
-      <c r="O13" s="5" t="n"/>
-      <c r="P13" s="5" t="n"/>
-      <c r="Q13" s="5" t="n"/>
-      <c r="R13" s="5" t="n"/>
+      <c r="N13" s="5" t="n">
+        <v>103.8</v>
+      </c>
+      <c r="O13" s="5" t="n">
+        <v>58.8</v>
+      </c>
+      <c r="P13" s="5" t="n">
+        <v>42.6</v>
+      </c>
+      <c r="Q13" s="5" t="n">
+        <v>28.2</v>
+      </c>
+      <c r="R13" s="5" t="n">
+        <v>4.1</v>
+      </c>
       <c r="AO13" t="inlineStr">
         <is>
           <t>Total operating income</t>
         </is>
+      </c>
+      <c r="AP13" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="AQ13" t="n">
+        <v>28.2</v>
+      </c>
+      <c r="AR13" t="n">
+        <v>42.6</v>
+      </c>
+      <c r="AS13" t="n">
+        <v>58.8</v>
+      </c>
+      <c r="AT13" t="n">
+        <v>103.8</v>
       </c>
       <c r="AU13" t="n">
         <v>166.1</v>
@@ -2915,15 +3040,40 @@
       <c r="M14" s="5" t="n">
         <v>-100.8</v>
       </c>
-      <c r="N14" s="5" t="n"/>
-      <c r="O14" s="5" t="n"/>
-      <c r="P14" s="5" t="n"/>
-      <c r="Q14" s="5" t="n"/>
-      <c r="R14" s="5" t="n"/>
+      <c r="N14" s="5" t="n">
+        <v>-69.5</v>
+      </c>
+      <c r="O14" s="5" t="n">
+        <v>-52.2</v>
+      </c>
+      <c r="P14" s="5" t="n">
+        <v>-42.6</v>
+      </c>
+      <c r="Q14" s="5" t="n">
+        <v>-35.6</v>
+      </c>
+      <c r="R14" s="5" t="n">
+        <v>-12.4</v>
+      </c>
       <c r="AO14" t="inlineStr">
         <is>
           <t>Administrative expenses</t>
         </is>
+      </c>
+      <c r="AP14" t="n">
+        <v>-12.4</v>
+      </c>
+      <c r="AQ14" t="n">
+        <v>-35.6</v>
+      </c>
+      <c r="AR14" t="n">
+        <v>-42.6</v>
+      </c>
+      <c r="AS14" t="n">
+        <v>-52.2</v>
+      </c>
+      <c r="AT14" t="n">
+        <v>-69.5</v>
       </c>
       <c r="AU14" t="n">
         <v>-100.8</v>
@@ -2999,15 +3149,40 @@
       <c r="M15" s="5" t="n">
         <v>39.7</v>
       </c>
-      <c r="N15" s="5" t="n"/>
-      <c r="O15" s="5" t="n"/>
-      <c r="P15" s="5" t="n"/>
-      <c r="Q15" s="5" t="n"/>
-      <c r="R15" s="5" t="n"/>
+      <c r="N15" s="5" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="O15" s="5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="P15" s="5" t="n">
+        <v>-0.9</v>
+      </c>
+      <c r="Q15" s="5" t="n">
+        <v>-8.800000000000001</v>
+      </c>
+      <c r="R15" s="5" t="n">
+        <v>-13</v>
+      </c>
       <c r="AO15" t="inlineStr">
         <is>
           <t>Profit after taxation</t>
         </is>
+      </c>
+      <c r="AP15" t="n">
+        <v>-13</v>
+      </c>
+      <c r="AQ15" t="n">
+        <v>-8.800000000000001</v>
+      </c>
+      <c r="AR15" t="n">
+        <v>-0.9</v>
+      </c>
+      <c r="AS15" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="AT15" t="n">
+        <v>23.4</v>
       </c>
       <c r="AU15" t="n">
         <v>39.7</v>
@@ -9622,7 +9797,7 @@
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>17050.8</v>
+        <v>19103.6</v>
       </c>
       <c r="C37" s="5" t="n">
         <v>18823.7</v>
@@ -10167,6 +10342,7 @@
 FY2016 &amp; FY2015: Full accounts for the year ended 31 December 2016, filed 11 May 2017, p.27 — https://find-and-update.company-information.service.gov.uk/company/00947662/filing-history/MzE3NTQ0MTgwOGFkaXF6a2N4/document?format=pdf&amp;download=0
 FY2014: Full accounts for the year ended 31 December 2015, filed 23 May 2016, p.77 (FY2014 comparative) — https://find-and-update.company-information.service.gov.uk/company/00947662/filing-history/MzE0OTEzMjU1M2FkaXF6a2N4/document?format=pdf&amp;download=0
 FY2017 has no standalone 12-month Statement of financial position: following the Bank's 2018 acquisition by FirstRand, its accounting reference date changed from 31 December to 30 June, producing one 18-month set of accounts (1 Jan 2017 - 30 Jun 2018, shown here as FY2018) instead of a normal FY2017 + FY2018 pair — FY2017 is left blank rather than estimated. FY2018's column is therefore an 18-month, not 12-month, snapshot; as a balance-sheet (point-in-time) statement this affects comparability less than the flow statements, but the period length difference should still be borne in mind when reading growth between FY2016 and FY2018.
+FY2025 TOTAL LIABILITIES CORRECTED 2026-10-08. This cell previously read 17,050.8, which was a transcription error, not a disclosed figure: the Bank's own Statement of financial position (FY2025 full accounts, p.54 of the filed PDF) prints Total liabilities of 19,103.6 (2024: 18,823.7). The error was surfaced by the column failing to balance three ways at once - the eight liability component rows above sum to 19,103.6, Total assets 20,618.2 less Total equity 1,514.6 is 19,103.6, and 17,050.8 + 1,514.6 came to 18,565.4 against a printed Total liabilities and equity of 20,618.2, an out-of-balance of 2,052.8. The source page was re-rendered at 300 dpi and read directly (the filed PDF is a scan with no text layer, so OCR was used for navigation only); every other figure in the FY2025 column was confirmed against that render and is unchanged. The likely mechanism is an eye-skip to the adjacent Customers' accounts line, which prints 17,047.6. The printed figure is reproduced; nothing is derived.
 Note: minor (£0.1m) rounding differences appear between the Total equity figure on the face of the Statement of financial position and the Statement of Changes in Equity's closing balance in some years (e.g. FY2021: £987.1m here vs £987.2m per the FY2021 accounts' own Statement of Changes in Equity) — both are presented exactly as disclosed in their respective source tables, not reconciled.
 Debt securities breakdown (measurement basis + issuer type), added as sub-rows directly beneath the 'Debt securities' line, sourced from the 'Debt securities' note of each year's own full statutory accounts (same Companies House filings/pages as above): FY2025/FY2024 — Note 12, p.79 of the FY2025 filing (https://find-and-update.company-information.service.gov.uk/company/00947662/filing-history/MzQ4NzM5MDg2MWFkaXF6a2N4/document?format=pdf&amp;download=0); FY2023/FY2022 — Note 11, p.78 of the FY2023 filing (https://find-and-update.company-information.service.gov.uk/company/00947662/filing-history/MzM5ODA0OTgzOWFkaXF6a2N4/document?format=pdf&amp;download=0); FY2021/FY2020 — Note 16, p.86 of the FY2021 filing (https://find-and-update.company-information.service.gov.uk/company/00947662/filing-history/MzMxODkyMzc2MWFkaXF6a2N4/document?format=pdf&amp;download=0). FY2020's 'UK Government gilts / treasury bills' sub-row (£235.0m) combines that year's own 'UK Government gilts and treasury bills' line (£188.9m) with a separate 'Treasury Bills' line (£46.1m) disclosed only as a FY2020 comparative in the FY2021 accounts. Sub-row sums reconcile to the 'Debt securities' total in every sourced year except FY2023 (£2,048.8m per the note vs £2,048.9m on the face of the Statement of financial position) and FY2022 (£2,339.3m vs £2,339.2m) — both are pre-existing £0.1m rounding artefacts in the Bank's own disclosures, not reconciled here. No equivalent note-level breakdown was sourced for FY2019 and earlier within this pass's scope (FY2020-FY2025 prioritised).
 HD-073 extension (FY2009-FY2013): sourced from the Bank's own full statutory accounts filed at Companies House, scanned/OCR'd (no text layer in the filed PDFs), prepared under old UK GAAP (not IFRS) as these pre-date the Bank's IFRS transition:

</xml_diff>